<commit_message>
Update Supplemental_Tables to account for new plots
</commit_message>
<xml_diff>
--- a/Supplemental_Tables/Table_S6.xlsx
+++ b/Supplemental_Tables/Table_S6.xlsx
@@ -5,38 +5,25 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kierstenruff/Documents/Collaborations/Su/2024/IDR_Basis_Set/2024_02/Figures/POLR/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kierstenruff/Documents/Collaborations/Su/2024/IDR_Basis_Set/2025_04/Supplemental_Tables/Finals/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B42EA2D-7E10-E147-8601-8AC6F579404E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A239FDAB-EB4A-D141-91F7-E0BB3FEAD7C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7160" yWindow="760" windowWidth="23000" windowHeight="20740" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11560" yWindow="760" windowWidth="23000" windowHeight="20740" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Fig_6B" sheetId="4" r:id="rId1"/>
-    <sheet name="Fig_6F" sheetId="2" r:id="rId2"/>
+    <sheet name="Fig_6D" sheetId="2" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Fig_6F!$A$1:$F$132</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Fig_6D!$A$1:$F$132</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="171">
-  <si>
-    <t>POLR1F IDR1</t>
-  </si>
-  <si>
-    <t>POLR1G IDR4</t>
-  </si>
-  <si>
-    <t>POLR1A IDR1</t>
-  </si>
-  <si>
-    <t>POLR2A IDR1</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="138">
   <si>
     <t>Gene</t>
   </si>
@@ -450,100 +437,13 @@
   </si>
   <si>
     <t>AFF2 IDR7</t>
-  </si>
-  <si>
-    <t>Sequence Features</t>
-  </si>
-  <si>
-    <t>pos-pos</t>
-  </si>
-  <si>
-    <t>pos-neg</t>
-  </si>
-  <si>
-    <t>pol-pos</t>
-  </si>
-  <si>
-    <t>N Patch</t>
-  </si>
-  <si>
-    <t>K Patch</t>
-  </si>
-  <si>
-    <t>Frac K</t>
-  </si>
-  <si>
-    <t>R/K Ratio</t>
-  </si>
-  <si>
-    <t>hyd-pos</t>
-  </si>
-  <si>
-    <t>pos-pro</t>
-  </si>
-  <si>
-    <t>hyd-pro</t>
-  </si>
-  <si>
-    <t>pro-pro</t>
-  </si>
-  <si>
-    <t>hyd-neg</t>
-  </si>
-  <si>
-    <t>neg-pro</t>
-  </si>
-  <si>
-    <t>E Patch</t>
-  </si>
-  <si>
-    <t>Frac E</t>
-  </si>
-  <si>
-    <t>pol-neg</t>
-  </si>
-  <si>
-    <t>Frac D+E</t>
-  </si>
-  <si>
-    <t>aro-aro</t>
-  </si>
-  <si>
-    <t>pol-aro</t>
-  </si>
-  <si>
-    <t>pol-pro</t>
-  </si>
-  <si>
-    <t>Frac Y</t>
-  </si>
-  <si>
-    <t>S Patch</t>
-  </si>
-  <si>
-    <t>aro-pro</t>
-  </si>
-  <si>
-    <t>pol-pol</t>
-  </si>
-  <si>
-    <t>Frac Aromatic</t>
-  </si>
-  <si>
-    <t>Frac S</t>
-  </si>
-  <si>
-    <t>Frac Aliphatic</t>
-  </si>
-  <si>
-    <t>Frac P</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -556,6 +456,13 @@
       <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -593,17 +500,79 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="7">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF58320"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF1E9AD9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF58320"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF1E9AD9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF58320"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF1E9AD9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FF1F8242"/>
+      <color rgb="FFF58320"/>
+      <color rgb="FF1E9AD9"/>
+      <color rgb="FFE43B34"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -899,385 +868,6 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:G30"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="3.1640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.83203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.1640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.83203125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B1" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="G1" s="1"/>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2" s="1">
-        <v>15</v>
-      </c>
-      <c r="B2" t="s">
-        <v>143</v>
-      </c>
-      <c r="C2">
-        <v>8.6912130739152875</v>
-      </c>
-      <c r="D2">
-        <v>7.0964901188400242</v>
-      </c>
-      <c r="E2">
-        <v>2.4097697157599161</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A3" s="1">
-        <v>16</v>
-      </c>
-      <c r="B3" t="s">
-        <v>144</v>
-      </c>
-      <c r="C3">
-        <v>8.5379255999914605</v>
-      </c>
-      <c r="D3">
-        <v>7.9008839170446006</v>
-      </c>
-      <c r="E3">
-        <v>4.2704882182517903</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A4" s="1">
-        <v>2</v>
-      </c>
-      <c r="B4" t="s">
-        <v>145</v>
-      </c>
-      <c r="C4">
-        <v>7.5317422896858206</v>
-      </c>
-      <c r="D4">
-        <v>5.1854287483593424</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A5" s="1">
-        <v>81</v>
-      </c>
-      <c r="B5" t="s">
-        <v>146</v>
-      </c>
-      <c r="C5">
-        <v>3.95172602916479</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A6" s="1">
-        <v>78</v>
-      </c>
-      <c r="B6" t="s">
-        <v>147</v>
-      </c>
-      <c r="C6">
-        <v>3.651848672424348</v>
-      </c>
-      <c r="D6">
-        <v>2.8704066986364212</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A7" s="1">
-        <v>44</v>
-      </c>
-      <c r="B7" t="s">
-        <v>148</v>
-      </c>
-      <c r="C7">
-        <v>2.8189650961096859</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A8" s="1">
-        <v>21</v>
-      </c>
-      <c r="B8" t="s">
-        <v>6</v>
-      </c>
-      <c r="C8">
-        <v>2.4621976233752441</v>
-      </c>
-      <c r="E8">
-        <v>3.2993076184605119</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A9" s="1">
-        <v>61</v>
-      </c>
-      <c r="B9" t="s">
-        <v>149</v>
-      </c>
-      <c r="C9">
-        <v>-2.2581109568702109</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A10" s="1">
-        <v>9</v>
-      </c>
-      <c r="B10" t="s">
-        <v>150</v>
-      </c>
-      <c r="D10">
-        <v>9.8573653824571466</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A11" s="1">
-        <v>19</v>
-      </c>
-      <c r="B11" t="s">
-        <v>151</v>
-      </c>
-      <c r="D11">
-        <v>8.4519087893759028</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A12" s="1">
-        <v>13</v>
-      </c>
-      <c r="B12" t="s">
-        <v>152</v>
-      </c>
-      <c r="D12">
-        <v>-3.2810248931287829</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A13" s="1">
-        <v>33</v>
-      </c>
-      <c r="B13" t="s">
-        <v>153</v>
-      </c>
-      <c r="D13">
-        <v>-2.9391667008166031</v>
-      </c>
-      <c r="F13">
-        <v>-7.0750059805988581</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A14" s="1">
-        <v>10</v>
-      </c>
-      <c r="B14" t="s">
-        <v>154</v>
-      </c>
-      <c r="D14">
-        <v>-2.906256539637524</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A15" s="1">
-        <v>24</v>
-      </c>
-      <c r="B15" t="s">
-        <v>155</v>
-      </c>
-      <c r="D15">
-        <v>-2.8924034665999701</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A16" s="1">
-        <v>73</v>
-      </c>
-      <c r="B16" t="s">
-        <v>156</v>
-      </c>
-      <c r="E16">
-        <v>2.3078959525978169</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A17" s="1">
-        <v>39</v>
-      </c>
-      <c r="B17" t="s">
-        <v>157</v>
-      </c>
-      <c r="E17">
-        <v>2.2240247378186719</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A18" s="1">
-        <v>3</v>
-      </c>
-      <c r="B18" t="s">
-        <v>158</v>
-      </c>
-      <c r="E18">
-        <v>2.162494286009832</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A19" s="1">
-        <v>57</v>
-      </c>
-      <c r="B19" t="s">
-        <v>159</v>
-      </c>
-      <c r="E19">
-        <v>2.1312033285413658</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A20" s="1">
-        <v>26</v>
-      </c>
-      <c r="B20" t="s">
-        <v>160</v>
-      </c>
-      <c r="F20">
-        <v>-7.8811920389992398</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A21" s="1">
-        <v>4</v>
-      </c>
-      <c r="B21" t="s">
-        <v>161</v>
-      </c>
-      <c r="F21">
-        <v>-7.1609601454156593</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A22" s="1">
-        <v>6</v>
-      </c>
-      <c r="B22" t="s">
-        <v>162</v>
-      </c>
-      <c r="F22">
-        <v>-6.8258087669737151</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A23" s="1">
-        <v>55</v>
-      </c>
-      <c r="B23" t="s">
-        <v>163</v>
-      </c>
-      <c r="F23">
-        <v>6.794134520118531</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A24" s="1">
-        <v>85</v>
-      </c>
-      <c r="B24" t="s">
-        <v>164</v>
-      </c>
-      <c r="F24">
-        <v>5.1425105105452058</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A25" s="1">
-        <v>28</v>
-      </c>
-      <c r="B25" t="s">
-        <v>165</v>
-      </c>
-      <c r="F25">
-        <v>-4.0194395026816219</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A26" s="1">
-        <v>0</v>
-      </c>
-      <c r="B26" t="s">
-        <v>166</v>
-      </c>
-      <c r="F26">
-        <v>-3.9071060353610099</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A27" s="1">
-        <v>60</v>
-      </c>
-      <c r="B27" t="s">
-        <v>167</v>
-      </c>
-      <c r="F27">
-        <v>3.7935570475830409</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A28" s="1">
-        <v>51</v>
-      </c>
-      <c r="B28" t="s">
-        <v>168</v>
-      </c>
-      <c r="F28">
-        <v>3.0176949354639548</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A29" s="1">
-        <v>59</v>
-      </c>
-      <c r="B29" t="s">
-        <v>169</v>
-      </c>
-      <c r="F29">
-        <v>-2.7566089891569061</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A30" s="1">
-        <v>48</v>
-      </c>
-      <c r="B30" t="s">
-        <v>170</v>
-      </c>
-      <c r="F30">
-        <v>2.2373201847316082</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:F132"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -1292,2210 +882,2210 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>4</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="1">
-        <v>93</v>
+        <v>47</v>
       </c>
       <c r="B2" t="s">
-        <v>104</v>
-      </c>
-      <c r="C2" t="s">
-        <v>13</v>
+        <v>54</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>6</v>
       </c>
       <c r="D2">
-        <v>0</v>
+        <v>12.703852167029639</v>
       </c>
       <c r="E2">
-        <v>98</v>
+        <v>2</v>
       </c>
       <c r="F2">
-        <v>223</v>
+        <v>131</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
-        <v>123</v>
+        <v>111</v>
       </c>
       <c r="B3" t="s">
-        <v>134</v>
-      </c>
-      <c r="C3" t="s">
-        <v>13</v>
+        <v>118</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>6</v>
       </c>
       <c r="D3">
-        <v>0</v>
+        <v>9.1373480382175245</v>
       </c>
       <c r="E3">
-        <v>94</v>
+        <v>67</v>
       </c>
       <c r="F3">
-        <v>172</v>
+        <v>1243</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
-        <v>19</v>
+        <v>43</v>
       </c>
       <c r="B4" t="s">
-        <v>30</v>
-      </c>
-      <c r="C4" t="s">
-        <v>13</v>
+        <v>50</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>6</v>
       </c>
       <c r="D4">
-        <v>0</v>
+        <v>8.6012553094958637</v>
       </c>
       <c r="E4">
-        <v>79</v>
+        <v>23</v>
       </c>
       <c r="F4">
-        <v>334</v>
+        <v>589</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
-        <v>33</v>
+        <v>116</v>
       </c>
       <c r="B5" t="s">
-        <v>44</v>
-      </c>
-      <c r="C5" t="s">
-        <v>13</v>
+        <v>123</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>6</v>
       </c>
       <c r="D5">
-        <v>0</v>
+        <v>7.3997255972020621</v>
       </c>
       <c r="E5">
-        <v>71</v>
+        <v>6</v>
       </c>
       <c r="F5">
-        <v>322</v>
+        <v>199</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
-        <v>111</v>
+        <v>66</v>
       </c>
       <c r="B6" t="s">
-        <v>122</v>
-      </c>
-      <c r="C6" t="s">
-        <v>10</v>
+        <v>73</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D6">
-        <v>9.1373480382175245</v>
+        <v>7.262249035589095</v>
       </c>
       <c r="E6">
-        <v>67</v>
+        <v>12</v>
       </c>
       <c r="F6">
-        <v>1243</v>
+        <v>92</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
-        <v>31</v>
+        <v>82</v>
       </c>
       <c r="B7" t="s">
-        <v>42</v>
-      </c>
-      <c r="C7" t="s">
-        <v>13</v>
+        <v>89</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>6</v>
       </c>
       <c r="D7">
-        <v>0</v>
+        <v>6.3660682604994943</v>
       </c>
       <c r="E7">
-        <v>53</v>
+        <v>5</v>
       </c>
       <c r="F7">
-        <v>406</v>
+        <v>127</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
-        <v>42</v>
+        <v>70</v>
       </c>
       <c r="B8" t="s">
-        <v>53</v>
-      </c>
-      <c r="C8" t="s">
-        <v>13</v>
+        <v>77</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>6</v>
       </c>
       <c r="D8">
-        <v>0</v>
+        <v>5.0918175034580182</v>
       </c>
       <c r="E8">
-        <v>49</v>
+        <v>2</v>
       </c>
       <c r="F8">
-        <v>158</v>
+        <v>129</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
-        <v>17</v>
+        <v>59</v>
       </c>
       <c r="B9" t="s">
-        <v>28</v>
-      </c>
-      <c r="C9" t="s">
-        <v>13</v>
+        <v>66</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D9">
-        <v>0</v>
+        <v>4.9088090544373264</v>
       </c>
       <c r="E9">
-        <v>42</v>
+        <v>14</v>
       </c>
       <c r="F9">
-        <v>366</v>
+        <v>301</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
-        <v>32</v>
+        <v>5</v>
       </c>
       <c r="B10" t="s">
-        <v>43</v>
-      </c>
-      <c r="C10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D10">
+        <v>4.8794322158906418</v>
+      </c>
+      <c r="E10">
         <v>13</v>
       </c>
-      <c r="D10">
-        <v>0</v>
-      </c>
-      <c r="E10">
-        <v>40</v>
-      </c>
       <c r="F10">
-        <v>228</v>
+        <v>248</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="1">
-        <v>79</v>
+        <v>8</v>
       </c>
       <c r="B11" t="s">
-        <v>90</v>
-      </c>
-      <c r="C11" t="s">
-        <v>13</v>
+        <v>15</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>6</v>
       </c>
       <c r="D11">
-        <v>1.255642593105738</v>
+        <v>4.6653570953300241</v>
       </c>
       <c r="E11">
-        <v>38</v>
+        <v>0.99999999999999989</v>
       </c>
       <c r="F11">
-        <v>833</v>
+        <v>107</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="1">
-        <v>53</v>
+        <v>23</v>
       </c>
       <c r="B12" t="s">
-        <v>64</v>
-      </c>
-      <c r="C12" t="s">
-        <v>13</v>
+        <v>30</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>6</v>
       </c>
       <c r="D12">
-        <v>0.2260744105017316</v>
+        <v>4.2123112982837299</v>
       </c>
       <c r="E12">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="F12">
-        <v>618</v>
+        <v>350</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" s="1">
-        <v>40</v>
+        <v>104</v>
       </c>
       <c r="B13" t="s">
-        <v>51</v>
-      </c>
-      <c r="C13" t="s">
-        <v>13</v>
+        <v>111</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>6</v>
       </c>
       <c r="D13">
-        <v>0</v>
+        <v>4.1647986302267643</v>
       </c>
       <c r="E13">
-        <v>33</v>
+        <v>14</v>
       </c>
       <c r="F13">
-        <v>202</v>
+        <v>348</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" s="1">
-        <v>18</v>
+        <v>78</v>
       </c>
       <c r="B14" t="s">
-        <v>29</v>
-      </c>
-      <c r="C14" t="s">
-        <v>13</v>
+        <v>85</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>6</v>
       </c>
       <c r="D14">
-        <v>0</v>
+        <v>3.8362616028192589</v>
       </c>
       <c r="E14">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="F14">
-        <v>213</v>
+        <v>289</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="1">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="B15" t="s">
-        <v>49</v>
-      </c>
-      <c r="C15" t="s">
-        <v>13</v>
+        <v>42</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>6</v>
       </c>
       <c r="D15">
-        <v>0</v>
+        <v>3.4119991771462912</v>
       </c>
       <c r="E15">
-        <v>31</v>
+        <v>6</v>
       </c>
       <c r="F15">
-        <v>322</v>
+        <v>111</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" s="1">
-        <v>12</v>
+        <v>105</v>
       </c>
       <c r="B16" t="s">
-        <v>23</v>
-      </c>
-      <c r="C16" t="s">
-        <v>13</v>
+        <v>112</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D16">
-        <v>0</v>
+        <v>3.298216319304649</v>
       </c>
       <c r="E16">
-        <v>26</v>
+        <v>5</v>
       </c>
       <c r="F16">
-        <v>149</v>
+        <v>97</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" s="1">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B17" t="s">
-        <v>54</v>
-      </c>
-      <c r="C17" t="s">
-        <v>10</v>
+        <v>48</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D17">
-        <v>8.6012553094958637</v>
+        <v>3.0578701079800221</v>
       </c>
       <c r="E17">
-        <v>23</v>
+        <v>5</v>
       </c>
       <c r="F17">
-        <v>589</v>
+        <v>88</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" s="1">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="B18" t="s">
-        <v>92</v>
-      </c>
-      <c r="C18" t="s">
-        <v>10</v>
+        <v>97</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>6</v>
       </c>
       <c r="D18">
-        <v>0.42435443184490701</v>
+        <v>2.7954531212338409</v>
       </c>
       <c r="E18">
-        <v>22</v>
+        <v>6.9999999999999991</v>
       </c>
       <c r="F18">
-        <v>364</v>
+        <v>187</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" s="1">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="B19" t="s">
-        <v>25</v>
-      </c>
-      <c r="C19" t="s">
         <v>13</v>
       </c>
+      <c r="C19" s="2" t="s">
+        <v>9</v>
+      </c>
       <c r="D19">
-        <v>0</v>
+        <v>2.6948601736134239</v>
       </c>
       <c r="E19">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="F19">
-        <v>196</v>
+        <v>58</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" s="1">
-        <v>9</v>
+        <v>98</v>
       </c>
       <c r="B20" t="s">
-        <v>20</v>
-      </c>
-      <c r="C20" t="s">
-        <v>10</v>
+        <v>105</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D20">
-        <v>0</v>
+        <v>2.6566375330570149</v>
       </c>
       <c r="E20">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="F20">
-        <v>235</v>
+        <v>181</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" s="1">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="B21" t="s">
-        <v>27</v>
-      </c>
-      <c r="C21" t="s">
-        <v>13</v>
+        <v>43</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>6</v>
       </c>
       <c r="D21">
-        <v>0</v>
+        <v>2.6500239639328731</v>
       </c>
       <c r="E21">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="F21">
-        <v>151</v>
+        <v>97</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" s="1">
-        <v>29</v>
+        <v>67</v>
       </c>
       <c r="B22" t="s">
-        <v>40</v>
-      </c>
-      <c r="C22" t="s">
-        <v>13</v>
+        <v>74</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D22">
-        <v>0</v>
+        <v>2.465257512248181</v>
       </c>
       <c r="E22">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="F22">
-        <v>629</v>
+        <v>81</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23" s="1">
-        <v>52</v>
+        <v>97</v>
       </c>
       <c r="B23" t="s">
-        <v>63</v>
-      </c>
-      <c r="C23" t="s">
-        <v>13</v>
+        <v>104</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>6</v>
       </c>
       <c r="D23">
-        <v>0</v>
+        <v>2.2543672941753572</v>
       </c>
       <c r="E23">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="F23">
-        <v>247</v>
+        <v>184</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" s="1">
-        <v>39</v>
+        <v>58</v>
       </c>
       <c r="B24" t="s">
-        <v>50</v>
-      </c>
-      <c r="C24" t="s">
-        <v>13</v>
+        <v>65</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D24">
-        <v>0</v>
+        <v>2.172414540608878</v>
       </c>
       <c r="E24">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="F24">
-        <v>165</v>
+        <v>187</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" s="1">
-        <v>69</v>
+        <v>4</v>
       </c>
       <c r="B25" t="s">
+        <v>11</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D25">
+        <v>2.16697827226829</v>
+      </c>
+      <c r="E25">
+        <v>4</v>
+      </c>
+      <c r="F25">
         <v>80</v>
-      </c>
-      <c r="C25" t="s">
-        <v>10</v>
-      </c>
-      <c r="D25">
-        <v>0.1895018763729262</v>
-      </c>
-      <c r="E25">
-        <v>17</v>
-      </c>
-      <c r="F25">
-        <v>355</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" s="1">
-        <v>73</v>
+        <v>13</v>
       </c>
       <c r="B26" t="s">
-        <v>84</v>
-      </c>
-      <c r="C26" t="s">
-        <v>13</v>
+        <v>20</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D26">
-        <v>1.842750881704087</v>
+        <v>1.898768304272791</v>
       </c>
       <c r="E26">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="F26">
-        <v>420</v>
+        <v>366</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27" s="1">
-        <v>124</v>
+        <v>73</v>
       </c>
       <c r="B27" t="s">
-        <v>135</v>
-      </c>
-      <c r="C27" t="s">
-        <v>13</v>
+        <v>80</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D27">
-        <v>0</v>
+        <v>1.842750881704087</v>
       </c>
       <c r="E27">
         <v>17</v>
       </c>
       <c r="F27">
-        <v>133</v>
+        <v>420</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A28" s="1">
-        <v>27</v>
+        <v>109</v>
       </c>
       <c r="B28" t="s">
-        <v>38</v>
-      </c>
-      <c r="C28" t="s">
-        <v>13</v>
+        <v>116</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>6</v>
       </c>
       <c r="D28">
-        <v>1.662120163731742</v>
+        <v>1.7658200271265549</v>
       </c>
       <c r="E28">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="F28">
-        <v>167</v>
+        <v>128</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A29" s="1">
-        <v>87</v>
+        <v>27</v>
       </c>
       <c r="B29" t="s">
-        <v>98</v>
-      </c>
-      <c r="C29" t="s">
-        <v>13</v>
+        <v>34</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D29">
-        <v>0</v>
+        <v>1.662120163731742</v>
       </c>
       <c r="E29">
         <v>15</v>
       </c>
       <c r="F29">
-        <v>328</v>
+        <v>167</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A30" s="1">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="B30" t="s">
-        <v>45</v>
-      </c>
-      <c r="C30" t="s">
-        <v>13</v>
+        <v>51</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D30">
-        <v>0</v>
+        <v>1.5957713228298589</v>
       </c>
       <c r="E30">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="F30">
-        <v>53</v>
+        <v>63</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A31" s="1">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B31" t="s">
-        <v>70</v>
-      </c>
-      <c r="C31" t="s">
-        <v>13</v>
+        <v>67</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D31">
-        <v>4.9088090544373264</v>
+        <v>1.4777290153168801</v>
       </c>
       <c r="E31">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F31">
-        <v>301</v>
+        <v>212</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A32" s="1">
-        <v>61</v>
+        <v>84</v>
       </c>
       <c r="B32" t="s">
+        <v>91</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D32">
+        <v>1.3636861773693369</v>
+      </c>
+      <c r="E32">
+        <v>2</v>
+      </c>
+      <c r="F32">
         <v>72</v>
-      </c>
-      <c r="C32" t="s">
-        <v>13</v>
-      </c>
-      <c r="D32">
-        <v>0</v>
-      </c>
-      <c r="E32">
-        <v>14</v>
-      </c>
-      <c r="F32">
-        <v>87</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A33" s="1">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="B33" t="s">
-        <v>115</v>
-      </c>
-      <c r="C33" t="s">
-        <v>10</v>
+        <v>114</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D33">
-        <v>4.1647986302267643</v>
+        <v>1.3518348393178721</v>
       </c>
       <c r="E33">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="F33">
-        <v>348</v>
+        <v>354</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A34" s="1">
-        <v>108</v>
+        <v>54</v>
       </c>
       <c r="B34" t="s">
-        <v>119</v>
-      </c>
-      <c r="C34" t="s">
-        <v>13</v>
+        <v>61</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D34">
-        <v>0</v>
+        <v>1.304364925955503</v>
       </c>
       <c r="E34">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="F34">
-        <v>112</v>
+        <v>102</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A35" s="1">
-        <v>0</v>
+        <v>79</v>
       </c>
       <c r="B35" t="s">
-        <v>9</v>
-      </c>
-      <c r="C35" t="s">
-        <v>10</v>
+        <v>86</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D35">
-        <v>0</v>
+        <v>1.255642593105738</v>
       </c>
       <c r="E35">
-        <v>13</v>
+        <v>38</v>
       </c>
       <c r="F35">
-        <v>142</v>
+        <v>833</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A36" s="1">
-        <v>5</v>
+        <v>56</v>
       </c>
       <c r="B36" t="s">
-        <v>16</v>
-      </c>
-      <c r="C36" t="s">
-        <v>13</v>
+        <v>63</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D36">
-        <v>4.8794322158906418</v>
+        <v>1.23299139795801</v>
       </c>
       <c r="E36">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F36">
-        <v>248</v>
+        <v>100</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A37" s="1">
-        <v>20</v>
+        <v>72</v>
       </c>
       <c r="B37" t="s">
-        <v>31</v>
-      </c>
-      <c r="C37" t="s">
-        <v>13</v>
+        <v>79</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D37">
-        <v>0</v>
+        <v>1.2310751411018901</v>
       </c>
       <c r="E37">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="F37">
-        <v>140</v>
+        <v>120</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A38" s="1">
-        <v>103</v>
+        <v>117</v>
       </c>
       <c r="B38" t="s">
-        <v>114</v>
-      </c>
-      <c r="C38" t="s">
-        <v>13</v>
+        <v>124</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>6</v>
       </c>
       <c r="D38">
-        <v>0</v>
+        <v>1.193721131834347</v>
       </c>
       <c r="E38">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="F38">
-        <v>165</v>
+        <v>93</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A39" s="1">
-        <v>3</v>
+        <v>120</v>
       </c>
       <c r="B39" t="s">
-        <v>14</v>
-      </c>
-      <c r="C39" t="s">
-        <v>13</v>
+        <v>127</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D39">
-        <v>0</v>
+        <v>1.1918215791420561</v>
       </c>
       <c r="E39">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="F39">
-        <v>79</v>
+        <v>87</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A40" s="1">
-        <v>7</v>
+        <v>127</v>
       </c>
       <c r="B40" t="s">
-        <v>18</v>
-      </c>
-      <c r="C40" t="s">
-        <v>13</v>
+        <v>134</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D40">
-        <v>0</v>
+        <v>1.106415483473163</v>
       </c>
       <c r="E40">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="F40">
-        <v>417</v>
+        <v>74</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A41" s="1">
-        <v>37</v>
+        <v>91</v>
       </c>
       <c r="B41" t="s">
-        <v>48</v>
-      </c>
-      <c r="C41" t="s">
-        <v>13</v>
+        <v>98</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D41">
-        <v>0</v>
+        <v>1.0403612371528641</v>
       </c>
       <c r="E41">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="F41">
-        <v>199</v>
+        <v>50</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A42" s="1">
-        <v>60</v>
+        <v>26</v>
       </c>
       <c r="B42" t="s">
-        <v>71</v>
-      </c>
-      <c r="C42" t="s">
-        <v>13</v>
+        <v>33</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>6</v>
       </c>
       <c r="D42">
-        <v>1.4777290153168801</v>
+        <v>0.97654408258811942</v>
       </c>
       <c r="E42">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="F42">
-        <v>212</v>
+        <v>171</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A43" s="1">
-        <v>66</v>
+        <v>128</v>
       </c>
       <c r="B43" t="s">
-        <v>77</v>
-      </c>
-      <c r="C43" t="s">
-        <v>13</v>
+        <v>135</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D43">
-        <v>7.262249035589095</v>
+        <v>0.89212433637271094</v>
       </c>
       <c r="E43">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="F43">
-        <v>92</v>
+        <v>87</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A44" s="1">
-        <v>23</v>
+        <v>92</v>
       </c>
       <c r="B44" t="s">
-        <v>34</v>
-      </c>
-      <c r="C44" t="s">
-        <v>10</v>
+        <v>99</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D44">
-        <v>4.2123112982837299</v>
+        <v>0.83910408072443454</v>
       </c>
       <c r="E44">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="F44">
-        <v>350</v>
+        <v>93</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A45" s="1">
-        <v>71</v>
+        <v>94</v>
       </c>
       <c r="B45" t="s">
-        <v>82</v>
-      </c>
-      <c r="C45" t="s">
-        <v>13</v>
+        <v>101</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D45">
-        <v>0</v>
+        <v>0.7932657348984451</v>
       </c>
       <c r="E45">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F45">
-        <v>70</v>
+        <v>98</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A46" s="1">
-        <v>30</v>
+        <v>114</v>
       </c>
       <c r="B46" t="s">
-        <v>41</v>
-      </c>
-      <c r="C46" t="s">
-        <v>13</v>
+        <v>121</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D46">
-        <v>0</v>
+        <v>0.76285517792187918</v>
       </c>
       <c r="E46">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="F46">
-        <v>79</v>
+        <v>74</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A47" s="1">
-        <v>56</v>
+        <v>129</v>
       </c>
       <c r="B47" t="s">
-        <v>67</v>
-      </c>
-      <c r="C47" t="s">
-        <v>13</v>
+        <v>136</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D47">
-        <v>1.23299139795801</v>
+        <v>0.70318197604183175</v>
       </c>
       <c r="E47">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F47">
-        <v>100</v>
+        <v>164</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A48" s="1">
-        <v>86</v>
+        <v>74</v>
       </c>
       <c r="B48" t="s">
-        <v>97</v>
-      </c>
-      <c r="C48" t="s">
-        <v>13</v>
+        <v>81</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D48">
-        <v>0</v>
+        <v>0.68991423123357676</v>
       </c>
       <c r="E48">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="F48">
-        <v>149</v>
+        <v>82</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A49" s="1">
-        <v>106</v>
+        <v>25</v>
       </c>
       <c r="B49" t="s">
-        <v>117</v>
-      </c>
-      <c r="C49" t="s">
-        <v>13</v>
+        <v>32</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D49">
-        <v>0</v>
+        <v>0.56461484944806117</v>
       </c>
       <c r="E49">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="F49">
-        <v>167</v>
+        <v>84</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A50" s="1">
-        <v>13</v>
+        <v>77</v>
       </c>
       <c r="B50" t="s">
-        <v>24</v>
-      </c>
-      <c r="C50" t="s">
-        <v>13</v>
+        <v>84</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>6</v>
       </c>
       <c r="D50">
-        <v>1.898768304272791</v>
+        <v>0.49344264139713467</v>
       </c>
       <c r="E50">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F50">
-        <v>366</v>
+        <v>88</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A51" s="1">
-        <v>26</v>
+        <v>57</v>
       </c>
       <c r="B51" t="s">
-        <v>37</v>
-      </c>
-      <c r="C51" t="s">
-        <v>10</v>
+        <v>64</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D51">
-        <v>0.97654408258811942</v>
+        <v>0.44028433351775331</v>
       </c>
       <c r="E51">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="F51">
-        <v>171</v>
+        <v>94</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A52" s="1">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="B52" t="s">
-        <v>89</v>
-      </c>
-      <c r="C52" t="s">
-        <v>10</v>
+        <v>88</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>6</v>
       </c>
       <c r="D52">
-        <v>3.8362616028192589</v>
+        <v>0.42435443184490701</v>
       </c>
       <c r="E52">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="F52">
-        <v>289</v>
+        <v>364</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A53" s="1">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B53" t="s">
-        <v>94</v>
-      </c>
-      <c r="C53" t="s">
-        <v>13</v>
+        <v>87</v>
+      </c>
+      <c r="C53" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D53">
-        <v>0</v>
+        <v>0.31096337755354819</v>
       </c>
       <c r="E53">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F53">
-        <v>149</v>
+        <v>342</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A54" s="1">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="B54" t="s">
-        <v>105</v>
-      </c>
-      <c r="C54" t="s">
-        <v>13</v>
+        <v>106</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>6</v>
       </c>
       <c r="D54">
-        <v>0.7932657348984451</v>
+        <v>0.30631500867905809</v>
       </c>
       <c r="E54">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="F54">
-        <v>98</v>
+        <v>93</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A55" s="1">
-        <v>113</v>
+        <v>101</v>
       </c>
       <c r="B55" t="s">
-        <v>124</v>
-      </c>
-      <c r="C55" t="s">
-        <v>13</v>
+        <v>108</v>
+      </c>
+      <c r="C55" s="2" t="s">
+        <v>6</v>
       </c>
       <c r="D55">
-        <v>0.17668253620412841</v>
+        <v>0.28376820996716362</v>
       </c>
       <c r="E55">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="F55">
-        <v>108</v>
+        <v>132</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A56" s="1">
-        <v>126</v>
+        <v>53</v>
       </c>
       <c r="B56" t="s">
-        <v>137</v>
-      </c>
-      <c r="C56" t="s">
-        <v>13</v>
+        <v>60</v>
+      </c>
+      <c r="C56" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D56">
-        <v>0</v>
+        <v>0.2260744105017316</v>
       </c>
       <c r="E56">
-        <v>9</v>
+        <v>36</v>
       </c>
       <c r="F56">
-        <v>103</v>
+        <v>618</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A57" s="1">
-        <v>2</v>
+        <v>69</v>
       </c>
       <c r="B57" t="s">
-        <v>12</v>
-      </c>
-      <c r="C57" t="s">
-        <v>13</v>
+        <v>76</v>
+      </c>
+      <c r="C57" s="2" t="s">
+        <v>6</v>
       </c>
       <c r="D57">
-        <v>0</v>
+        <v>0.1895018763729262</v>
       </c>
       <c r="E57">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="F57">
-        <v>101</v>
+        <v>355</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A58" s="1">
-        <v>49</v>
+        <v>113</v>
       </c>
       <c r="B58" t="s">
-        <v>60</v>
-      </c>
-      <c r="C58" t="s">
-        <v>13</v>
+        <v>120</v>
+      </c>
+      <c r="C58" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D58">
-        <v>0</v>
+        <v>0.17668253620412841</v>
       </c>
       <c r="E58">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F58">
-        <v>156</v>
+        <v>108</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A59" s="1">
-        <v>62</v>
+        <v>93</v>
       </c>
       <c r="B59" t="s">
-        <v>73</v>
-      </c>
-      <c r="C59" t="s">
-        <v>13</v>
+        <v>100</v>
+      </c>
+      <c r="C59" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D59">
-        <v>-4.8038020259127602E-2</v>
+        <v>0</v>
       </c>
       <c r="E59">
-        <v>8</v>
+        <v>98</v>
       </c>
       <c r="F59">
-        <v>141</v>
+        <v>223</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A60" s="1">
-        <v>72</v>
+        <v>123</v>
       </c>
       <c r="B60" t="s">
-        <v>83</v>
-      </c>
-      <c r="C60" t="s">
-        <v>13</v>
+        <v>130</v>
+      </c>
+      <c r="C60" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D60">
-        <v>1.2310751411018901</v>
+        <v>0</v>
       </c>
       <c r="E60">
-        <v>8</v>
+        <v>94</v>
       </c>
       <c r="F60">
-        <v>120</v>
+        <v>172</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A61" s="1">
-        <v>77</v>
+        <v>19</v>
       </c>
       <c r="B61" t="s">
-        <v>88</v>
-      </c>
-      <c r="C61" t="s">
-        <v>10</v>
+        <v>26</v>
+      </c>
+      <c r="C61" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D61">
-        <v>0.49344264139713467</v>
+        <v>0</v>
       </c>
       <c r="E61">
-        <v>8</v>
+        <v>79</v>
       </c>
       <c r="F61">
-        <v>88</v>
+        <v>334</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A62" s="1">
-        <v>97</v>
+        <v>33</v>
       </c>
       <c r="B62" t="s">
-        <v>108</v>
-      </c>
-      <c r="C62" t="s">
-        <v>10</v>
+        <v>40</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D62">
-        <v>2.2543672941753572</v>
+        <v>0</v>
       </c>
       <c r="E62">
-        <v>8</v>
+        <v>71</v>
       </c>
       <c r="F62">
-        <v>184</v>
+        <v>322</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A63" s="1">
-        <v>55</v>
+        <v>31</v>
       </c>
       <c r="B63" t="s">
-        <v>66</v>
-      </c>
-      <c r="C63" t="s">
-        <v>13</v>
+        <v>38</v>
+      </c>
+      <c r="C63" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D63">
         <v>0</v>
       </c>
       <c r="E63">
-        <v>7.0000000000000009</v>
+        <v>53</v>
       </c>
       <c r="F63">
-        <v>213</v>
+        <v>406</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A64" s="1">
-        <v>102</v>
+        <v>42</v>
       </c>
       <c r="B64" t="s">
-        <v>113</v>
-      </c>
-      <c r="C64" t="s">
-        <v>13</v>
+        <v>49</v>
+      </c>
+      <c r="C64" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D64">
         <v>0</v>
       </c>
       <c r="E64">
-        <v>7.0000000000000009</v>
+        <v>49</v>
       </c>
       <c r="F64">
-        <v>169</v>
+        <v>158</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A65" s="1">
-        <v>112</v>
+        <v>17</v>
       </c>
       <c r="B65" t="s">
-        <v>123</v>
-      </c>
-      <c r="C65" t="s">
-        <v>10</v>
+        <v>24</v>
+      </c>
+      <c r="C65" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D65">
-        <v>-0.66393459056578163</v>
+        <v>0</v>
       </c>
       <c r="E65">
-        <v>7.0000000000000009</v>
+        <v>42</v>
       </c>
       <c r="F65">
-        <v>169</v>
+        <v>366</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A66" s="1">
-        <v>15</v>
+        <v>32</v>
       </c>
       <c r="B66" t="s">
-        <v>26</v>
-      </c>
-      <c r="C66" t="s">
-        <v>13</v>
+        <v>39</v>
+      </c>
+      <c r="C66" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D66">
         <v>0</v>
       </c>
       <c r="E66">
-        <v>7</v>
+        <v>40</v>
       </c>
       <c r="F66">
-        <v>75</v>
+        <v>228</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A67" s="1">
-        <v>21</v>
+        <v>40</v>
       </c>
       <c r="B67" t="s">
-        <v>32</v>
-      </c>
-      <c r="C67" t="s">
-        <v>13</v>
+        <v>47</v>
+      </c>
+      <c r="C67" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D67">
         <v>0</v>
       </c>
       <c r="E67">
-        <v>7</v>
+        <v>33</v>
       </c>
       <c r="F67">
-        <v>216</v>
+        <v>202</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A68" s="1">
-        <v>44</v>
+        <v>18</v>
       </c>
       <c r="B68" t="s">
-        <v>55</v>
-      </c>
-      <c r="C68" t="s">
-        <v>13</v>
+        <v>25</v>
+      </c>
+      <c r="C68" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D68">
-        <v>1.5957713228298589</v>
+        <v>0</v>
       </c>
       <c r="E68">
-        <v>7</v>
+        <v>32</v>
       </c>
       <c r="F68">
-        <v>63</v>
+        <v>213</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A69" s="1">
+        <v>38</v>
+      </c>
+      <c r="B69" t="s">
         <v>45</v>
       </c>
-      <c r="B69" t="s">
-        <v>56</v>
-      </c>
-      <c r="C69" t="s">
-        <v>13</v>
+      <c r="C69" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D69">
         <v>0</v>
       </c>
       <c r="E69">
-        <v>7</v>
+        <v>31</v>
       </c>
       <c r="F69">
-        <v>119</v>
+        <v>322</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A70" s="1">
-        <v>80</v>
+        <v>12</v>
       </c>
       <c r="B70" t="s">
-        <v>91</v>
-      </c>
-      <c r="C70" t="s">
-        <v>13</v>
+        <v>19</v>
+      </c>
+      <c r="C70" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D70">
-        <v>0.31096337755354819</v>
+        <v>0</v>
       </c>
       <c r="E70">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="F70">
-        <v>342</v>
+        <v>149</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A71" s="1">
-        <v>96</v>
+        <v>14</v>
       </c>
       <c r="B71" t="s">
-        <v>107</v>
-      </c>
-      <c r="C71" t="s">
-        <v>13</v>
+        <v>21</v>
+      </c>
+      <c r="C71" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D71">
         <v>0</v>
       </c>
       <c r="E71">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="F71">
-        <v>99</v>
+        <v>196</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A72" s="1">
-        <v>90</v>
+        <v>9</v>
       </c>
       <c r="B72" t="s">
-        <v>101</v>
-      </c>
-      <c r="C72" t="s">
-        <v>10</v>
+        <v>16</v>
+      </c>
+      <c r="C72" s="2" t="s">
+        <v>6</v>
       </c>
       <c r="D72">
-        <v>2.7954531212338409</v>
+        <v>0</v>
       </c>
       <c r="E72">
-        <v>6.9999999999999991</v>
+        <v>19</v>
       </c>
       <c r="F72">
-        <v>187</v>
+        <v>235</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A73" s="1">
-        <v>35</v>
+        <v>16</v>
       </c>
       <c r="B73" t="s">
-        <v>46</v>
-      </c>
-      <c r="C73" t="s">
-        <v>10</v>
+        <v>23</v>
+      </c>
+      <c r="C73" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D73">
-        <v>3.4119991771462912</v>
+        <v>0</v>
       </c>
       <c r="E73">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="F73">
-        <v>111</v>
+        <v>151</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A74" s="1">
-        <v>67</v>
+        <v>29</v>
       </c>
       <c r="B74" t="s">
-        <v>78</v>
-      </c>
-      <c r="C74" t="s">
-        <v>13</v>
+        <v>36</v>
+      </c>
+      <c r="C74" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D74">
-        <v>2.465257512248181</v>
+        <v>0</v>
       </c>
       <c r="E74">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="F74">
-        <v>81</v>
+        <v>629</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A75" s="1">
-        <v>98</v>
+        <v>52</v>
       </c>
       <c r="B75" t="s">
-        <v>109</v>
-      </c>
-      <c r="C75" t="s">
-        <v>13</v>
+        <v>59</v>
+      </c>
+      <c r="C75" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D75">
-        <v>2.6566375330570149</v>
+        <v>0</v>
       </c>
       <c r="E75">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="F75">
-        <v>181</v>
+        <v>247</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A76" s="1">
-        <v>115</v>
+        <v>39</v>
       </c>
       <c r="B76" t="s">
-        <v>126</v>
-      </c>
-      <c r="C76" t="s">
-        <v>10</v>
+        <v>46</v>
+      </c>
+      <c r="C76" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D76">
         <v>0</v>
       </c>
       <c r="E76">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="F76">
-        <v>93</v>
+        <v>165</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A77" s="1">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="B77" t="s">
-        <v>127</v>
-      </c>
-      <c r="C77" t="s">
-        <v>10</v>
+        <v>131</v>
+      </c>
+      <c r="C77" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D77">
-        <v>7.3997255972020621</v>
+        <v>0</v>
       </c>
       <c r="E77">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="F77">
-        <v>199</v>
+        <v>133</v>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A78" s="1">
-        <v>122</v>
+        <v>87</v>
       </c>
       <c r="B78" t="s">
-        <v>133</v>
-      </c>
-      <c r="C78" t="s">
-        <v>13</v>
+        <v>94</v>
+      </c>
+      <c r="C78" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D78">
         <v>0</v>
       </c>
       <c r="E78">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="F78">
-        <v>78</v>
+        <v>328</v>
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A79" s="1">
-        <v>129</v>
+        <v>34</v>
       </c>
       <c r="B79" t="s">
-        <v>140</v>
-      </c>
-      <c r="C79" t="s">
-        <v>13</v>
+        <v>41</v>
+      </c>
+      <c r="C79" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D79">
-        <v>0.70318197604183175</v>
+        <v>0</v>
       </c>
       <c r="E79">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="F79">
-        <v>164</v>
+        <v>53</v>
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A80" s="1">
-        <v>25</v>
+        <v>61</v>
       </c>
       <c r="B80" t="s">
-        <v>36</v>
-      </c>
-      <c r="C80" t="s">
-        <v>13</v>
+        <v>68</v>
+      </c>
+      <c r="C80" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D80">
-        <v>0.56461484944806117</v>
+        <v>0</v>
       </c>
       <c r="E80">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="F80">
-        <v>84</v>
+        <v>87</v>
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A81" s="1">
-        <v>41</v>
+        <v>108</v>
       </c>
       <c r="B81" t="s">
-        <v>52</v>
-      </c>
-      <c r="C81" t="s">
-        <v>13</v>
+        <v>115</v>
+      </c>
+      <c r="C81" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D81">
-        <v>3.0578701079800221</v>
+        <v>0</v>
       </c>
       <c r="E81">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="F81">
-        <v>88</v>
+        <v>112</v>
       </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A82" s="1">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="B82" t="s">
-        <v>61</v>
-      </c>
-      <c r="C82" t="s">
+        <v>5</v>
+      </c>
+      <c r="C82" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D82">
+        <v>0</v>
+      </c>
+      <c r="E82">
         <v>13</v>
       </c>
-      <c r="D82">
-        <v>0</v>
-      </c>
-      <c r="E82">
-        <v>5</v>
-      </c>
       <c r="F82">
-        <v>98</v>
+        <v>142</v>
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A83" s="1">
-        <v>63</v>
+        <v>20</v>
       </c>
       <c r="B83" t="s">
-        <v>74</v>
-      </c>
-      <c r="C83" t="s">
+        <v>27</v>
+      </c>
+      <c r="C83" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D83">
+        <v>0</v>
+      </c>
+      <c r="E83">
         <v>13</v>
       </c>
-      <c r="D83">
-        <v>0</v>
-      </c>
-      <c r="E83">
-        <v>5</v>
-      </c>
       <c r="F83">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A84" s="1">
-        <v>82</v>
+        <v>103</v>
       </c>
       <c r="B84" t="s">
-        <v>93</v>
-      </c>
-      <c r="C84" t="s">
-        <v>10</v>
+        <v>110</v>
+      </c>
+      <c r="C84" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D84">
-        <v>6.3660682604994943</v>
+        <v>0</v>
       </c>
       <c r="E84">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="F84">
-        <v>127</v>
+        <v>165</v>
       </c>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A85" s="1">
-        <v>88</v>
+        <v>3</v>
       </c>
       <c r="B85" t="s">
-        <v>99</v>
-      </c>
-      <c r="C85" t="s">
-        <v>13</v>
+        <v>10</v>
+      </c>
+      <c r="C85" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D85">
-        <v>-0.87195005133563086</v>
+        <v>0</v>
       </c>
       <c r="E85">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="F85">
-        <v>120</v>
+        <v>79</v>
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A86" s="1">
-        <v>89</v>
+        <v>7</v>
       </c>
       <c r="B86" t="s">
-        <v>100</v>
-      </c>
-      <c r="C86" t="s">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="C86" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D86">
-        <v>-0.61584370402419808</v>
+        <v>0</v>
       </c>
       <c r="E86">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="F86">
-        <v>55</v>
+        <v>417</v>
       </c>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A87" s="1">
-        <v>101</v>
+        <v>37</v>
       </c>
       <c r="B87" t="s">
-        <v>112</v>
-      </c>
-      <c r="C87" t="s">
-        <v>10</v>
+        <v>44</v>
+      </c>
+      <c r="C87" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D87">
-        <v>0.28376820996716362</v>
+        <v>0</v>
       </c>
       <c r="E87">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="F87">
-        <v>132</v>
+        <v>199</v>
       </c>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A88" s="1">
-        <v>105</v>
+        <v>71</v>
       </c>
       <c r="B88" t="s">
-        <v>116</v>
-      </c>
-      <c r="C88" t="s">
-        <v>13</v>
+        <v>78</v>
+      </c>
+      <c r="C88" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D88">
-        <v>3.298216319304649</v>
+        <v>0</v>
       </c>
       <c r="E88">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="F88">
-        <v>97</v>
+        <v>70</v>
       </c>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A89" s="1">
-        <v>125</v>
+        <v>30</v>
       </c>
       <c r="B89" t="s">
-        <v>136</v>
-      </c>
-      <c r="C89" t="s">
-        <v>13</v>
+        <v>37</v>
+      </c>
+      <c r="C89" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D89">
         <v>0</v>
       </c>
       <c r="E89">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F89">
-        <v>193</v>
+        <v>79</v>
       </c>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A90" s="1">
-        <v>4</v>
+        <v>86</v>
       </c>
       <c r="B90" t="s">
-        <v>15</v>
-      </c>
-      <c r="C90" t="s">
-        <v>13</v>
+        <v>93</v>
+      </c>
+      <c r="C90" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D90">
-        <v>2.16697827226829</v>
+        <v>0</v>
       </c>
       <c r="E90">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="F90">
-        <v>80</v>
+        <v>149</v>
       </c>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A91" s="1">
-        <v>54</v>
+        <v>106</v>
       </c>
       <c r="B91" t="s">
-        <v>65</v>
-      </c>
-      <c r="C91" t="s">
-        <v>13</v>
+        <v>113</v>
+      </c>
+      <c r="C91" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D91">
-        <v>1.304364925955503</v>
+        <v>0</v>
       </c>
       <c r="E91">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="F91">
-        <v>102</v>
+        <v>167</v>
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A92" s="1">
-        <v>58</v>
+        <v>83</v>
       </c>
       <c r="B92" t="s">
-        <v>69</v>
-      </c>
-      <c r="C92" t="s">
-        <v>13</v>
+        <v>90</v>
+      </c>
+      <c r="C92" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D92">
-        <v>2.172414540608878</v>
+        <v>0</v>
       </c>
       <c r="E92">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="F92">
-        <v>187</v>
+        <v>149</v>
       </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A93" s="1">
-        <v>68</v>
+        <v>126</v>
       </c>
       <c r="B93" t="s">
-        <v>79</v>
-      </c>
-      <c r="C93" t="s">
-        <v>10</v>
+        <v>133</v>
+      </c>
+      <c r="C93" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D93">
-        <v>-1.827019897327971</v>
+        <v>0</v>
       </c>
       <c r="E93">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="F93">
-        <v>63</v>
+        <v>103</v>
       </c>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A94" s="1">
-        <v>75</v>
+        <v>2</v>
       </c>
       <c r="B94" t="s">
-        <v>86</v>
-      </c>
-      <c r="C94" t="s">
-        <v>13</v>
+        <v>8</v>
+      </c>
+      <c r="C94" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D94">
         <v>0</v>
       </c>
       <c r="E94">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="F94">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A95" s="1">
-        <v>76</v>
+        <v>49</v>
       </c>
       <c r="B95" t="s">
-        <v>87</v>
-      </c>
-      <c r="C95" t="s">
-        <v>10</v>
+        <v>56</v>
+      </c>
+      <c r="C95" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D95">
-        <v>-0.29438126778694468</v>
+        <v>0</v>
       </c>
       <c r="E95">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="F95">
-        <v>67</v>
+        <v>156</v>
       </c>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A96" s="1">
-        <v>85</v>
+        <v>55</v>
       </c>
       <c r="B96" t="s">
-        <v>96</v>
-      </c>
-      <c r="C96" t="s">
-        <v>13</v>
+        <v>62</v>
+      </c>
+      <c r="C96" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D96">
         <v>0</v>
       </c>
       <c r="E96">
-        <v>4</v>
+        <v>7.0000000000000009</v>
       </c>
       <c r="F96">
-        <v>98</v>
+        <v>213</v>
       </c>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A97" s="1">
-        <v>91</v>
+        <v>102</v>
       </c>
       <c r="B97" t="s">
-        <v>102</v>
-      </c>
-      <c r="C97" t="s">
-        <v>13</v>
+        <v>109</v>
+      </c>
+      <c r="C97" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D97">
-        <v>1.0403612371528641</v>
+        <v>0</v>
       </c>
       <c r="E97">
-        <v>4</v>
+        <v>7.0000000000000009</v>
       </c>
       <c r="F97">
-        <v>50</v>
+        <v>169</v>
       </c>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A98" s="1">
-        <v>99</v>
+        <v>15</v>
       </c>
       <c r="B98" t="s">
-        <v>110</v>
-      </c>
-      <c r="C98" t="s">
-        <v>10</v>
+        <v>22</v>
+      </c>
+      <c r="C98" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D98">
-        <v>0.30631500867905809</v>
+        <v>0</v>
       </c>
       <c r="E98">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="F98">
-        <v>93</v>
+        <v>75</v>
       </c>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A99" s="1">
-        <v>117</v>
+        <v>21</v>
       </c>
       <c r="B99" t="s">
-        <v>128</v>
-      </c>
-      <c r="C99" t="s">
-        <v>10</v>
+        <v>28</v>
+      </c>
+      <c r="C99" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D99">
-        <v>1.193721131834347</v>
+        <v>0</v>
       </c>
       <c r="E99">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="F99">
-        <v>93</v>
+        <v>216</v>
       </c>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A100" s="1">
-        <v>127</v>
+        <v>45</v>
       </c>
       <c r="B100" t="s">
-        <v>138</v>
-      </c>
-      <c r="C100" t="s">
-        <v>13</v>
+        <v>52</v>
+      </c>
+      <c r="C100" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D100">
-        <v>1.106415483473163</v>
+        <v>0</v>
       </c>
       <c r="E100">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="F100">
-        <v>74</v>
+        <v>119</v>
       </c>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A101" s="1">
-        <v>128</v>
+        <v>96</v>
       </c>
       <c r="B101" t="s">
-        <v>139</v>
-      </c>
-      <c r="C101" t="s">
-        <v>13</v>
+        <v>103</v>
+      </c>
+      <c r="C101" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D101">
-        <v>0.89212433637271094</v>
+        <v>0</v>
       </c>
       <c r="E101">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="F101">
-        <v>87</v>
+        <v>99</v>
       </c>
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A102" s="1">
-        <v>22</v>
+        <v>115</v>
       </c>
       <c r="B102" t="s">
-        <v>33</v>
-      </c>
-      <c r="C102" t="s">
-        <v>10</v>
+        <v>122</v>
+      </c>
+      <c r="C102" s="2" t="s">
+        <v>6</v>
       </c>
       <c r="D102">
-        <v>-0.64182248254319685</v>
+        <v>0</v>
       </c>
       <c r="E102">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F102">
-        <v>204</v>
+        <v>93</v>
       </c>
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A103" s="1">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="B103" t="s">
-        <v>106</v>
-      </c>
-      <c r="C103" t="s">
-        <v>13</v>
+        <v>129</v>
+      </c>
+      <c r="C103" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D103">
         <v>0</v>
       </c>
       <c r="E103">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F103">
-        <v>107</v>
+        <v>78</v>
       </c>
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A104" s="1">
-        <v>118</v>
+        <v>50</v>
       </c>
       <c r="B104" t="s">
-        <v>129</v>
-      </c>
-      <c r="C104" t="s">
-        <v>13</v>
+        <v>57</v>
+      </c>
+      <c r="C104" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D104">
         <v>0</v>
       </c>
       <c r="E104">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F104">
-        <v>134</v>
+        <v>98</v>
       </c>
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A105" s="1">
-        <v>6</v>
+        <v>63</v>
       </c>
       <c r="B105" t="s">
-        <v>17</v>
-      </c>
-      <c r="C105" t="s">
-        <v>13</v>
+        <v>70</v>
+      </c>
+      <c r="C105" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D105">
-        <v>2.6948601736134239</v>
+        <v>0</v>
       </c>
       <c r="E105">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F105">
-        <v>58</v>
+        <v>141</v>
       </c>
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A106" s="1">
-        <v>10</v>
+        <v>125</v>
       </c>
       <c r="B106" t="s">
-        <v>21</v>
-      </c>
-      <c r="C106" t="s">
-        <v>13</v>
+        <v>132</v>
+      </c>
+      <c r="C106" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D106">
         <v>0</v>
       </c>
       <c r="E106">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F106">
-        <v>73</v>
+        <v>193</v>
       </c>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A107" s="1">
-        <v>28</v>
+        <v>75</v>
       </c>
       <c r="B107" t="s">
-        <v>39</v>
-      </c>
-      <c r="C107" t="s">
-        <v>13</v>
+        <v>82</v>
+      </c>
+      <c r="C107" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D107">
-        <v>-0.51980146313749753</v>
+        <v>0</v>
       </c>
       <c r="E107">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F107">
-        <v>75</v>
+        <v>100</v>
       </c>
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A108" s="1">
-        <v>46</v>
+        <v>85</v>
       </c>
       <c r="B108" t="s">
-        <v>57</v>
-      </c>
-      <c r="C108" t="s">
-        <v>13</v>
+        <v>92</v>
+      </c>
+      <c r="C108" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D108">
-        <v>-0.34918308632545703</v>
+        <v>0</v>
       </c>
       <c r="E108">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F108">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A109" s="1">
-        <v>47</v>
+        <v>95</v>
       </c>
       <c r="B109" t="s">
-        <v>58</v>
-      </c>
-      <c r="C109" t="s">
-        <v>10</v>
+        <v>102</v>
+      </c>
+      <c r="C109" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D109">
-        <v>12.703852167029639</v>
+        <v>0</v>
       </c>
       <c r="E109">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F109">
-        <v>131</v>
+        <v>107</v>
       </c>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A110" s="1">
-        <v>57</v>
+        <v>118</v>
       </c>
       <c r="B110" t="s">
-        <v>68</v>
-      </c>
-      <c r="C110" t="s">
-        <v>13</v>
+        <v>125</v>
+      </c>
+      <c r="C110" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D110">
-        <v>0.44028433351775331</v>
+        <v>0</v>
       </c>
       <c r="E110">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F110">
-        <v>94</v>
+        <v>134</v>
       </c>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A111" s="1">
-        <v>64</v>
+        <v>10</v>
       </c>
       <c r="B111" t="s">
-        <v>75</v>
-      </c>
-      <c r="C111" t="s">
-        <v>13</v>
+        <v>17</v>
+      </c>
+      <c r="C111" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D111">
         <v>0</v>
@@ -3504,435 +3094,465 @@
         <v>2</v>
       </c>
       <c r="F111">
-        <v>78</v>
+        <v>73</v>
       </c>
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A112" s="1">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="B112" t="s">
-        <v>81</v>
-      </c>
-      <c r="C112" t="s">
-        <v>10</v>
+        <v>71</v>
+      </c>
+      <c r="C112" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D112">
-        <v>5.0918175034580182</v>
+        <v>0</v>
       </c>
       <c r="E112">
         <v>2</v>
       </c>
       <c r="F112">
-        <v>129</v>
+        <v>78</v>
       </c>
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A113" s="1">
-        <v>74</v>
+        <v>119</v>
       </c>
       <c r="B113" t="s">
-        <v>85</v>
-      </c>
-      <c r="C113" t="s">
-        <v>13</v>
+        <v>126</v>
+      </c>
+      <c r="C113" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D113">
-        <v>0.68991423123357676</v>
+        <v>0</v>
       </c>
       <c r="E113">
         <v>2</v>
       </c>
       <c r="F113">
-        <v>82</v>
+        <v>67</v>
       </c>
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A114" s="1">
-        <v>84</v>
+        <v>121</v>
       </c>
       <c r="B114" t="s">
-        <v>95</v>
-      </c>
-      <c r="C114" t="s">
-        <v>13</v>
+        <v>128</v>
+      </c>
+      <c r="C114" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D114">
-        <v>1.3636861773693369</v>
+        <v>0</v>
       </c>
       <c r="E114">
         <v>2</v>
       </c>
       <c r="F114">
-        <v>72</v>
+        <v>75</v>
       </c>
     </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A115" s="1">
-        <v>100</v>
+        <v>130</v>
       </c>
       <c r="B115" t="s">
-        <v>111</v>
-      </c>
-      <c r="C115" t="s">
-        <v>10</v>
+        <v>137</v>
+      </c>
+      <c r="C115" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D115">
-        <v>-0.13718772674175489</v>
+        <v>0</v>
       </c>
       <c r="E115">
         <v>2</v>
       </c>
       <c r="F115">
-        <v>66</v>
+        <v>84</v>
       </c>
     </row>
     <row r="116" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A116" s="1">
-        <v>109</v>
+        <v>24</v>
       </c>
       <c r="B116" t="s">
-        <v>120</v>
-      </c>
-      <c r="C116" t="s">
-        <v>10</v>
+        <v>31</v>
+      </c>
+      <c r="C116" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D116">
-        <v>1.7658200271265549</v>
+        <v>0</v>
       </c>
       <c r="E116">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F116">
-        <v>128</v>
+        <v>57</v>
       </c>
     </row>
     <row r="117" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A117" s="1">
-        <v>114</v>
+        <v>48</v>
       </c>
       <c r="B117" t="s">
-        <v>125</v>
-      </c>
-      <c r="C117" t="s">
-        <v>13</v>
+        <v>55</v>
+      </c>
+      <c r="C117" s="2" t="s">
+        <v>6</v>
       </c>
       <c r="D117">
-        <v>0.76285517792187918</v>
+        <v>0</v>
       </c>
       <c r="E117">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F117">
-        <v>74</v>
+        <v>89</v>
       </c>
     </row>
     <row r="118" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A118" s="1">
-        <v>119</v>
+        <v>11</v>
       </c>
       <c r="B118" t="s">
-        <v>130</v>
-      </c>
-      <c r="C118" t="s">
-        <v>13</v>
+        <v>18</v>
+      </c>
+      <c r="C118" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D118">
         <v>0</v>
       </c>
       <c r="E118">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F118">
-        <v>67</v>
+        <v>93</v>
       </c>
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A119" s="1">
-        <v>121</v>
+        <v>51</v>
       </c>
       <c r="B119" t="s">
-        <v>132</v>
-      </c>
-      <c r="C119" t="s">
-        <v>13</v>
+        <v>58</v>
+      </c>
+      <c r="C119" s="2" t="s">
+        <v>6</v>
       </c>
       <c r="D119">
         <v>0</v>
       </c>
       <c r="E119">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F119">
-        <v>75</v>
+        <v>56</v>
       </c>
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A120" s="1">
-        <v>130</v>
+        <v>62</v>
       </c>
       <c r="B120" t="s">
+        <v>69</v>
+      </c>
+      <c r="C120" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D120">
+        <v>-4.8038020259127602E-2</v>
+      </c>
+      <c r="E120">
+        <v>8</v>
+      </c>
+      <c r="F120">
         <v>141</v>
-      </c>
-      <c r="C120" t="s">
-        <v>13</v>
-      </c>
-      <c r="D120">
-        <v>0</v>
-      </c>
-      <c r="E120">
-        <v>2</v>
-      </c>
-      <c r="F120">
-        <v>84</v>
       </c>
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A121" s="1">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="B121" t="s">
-        <v>11</v>
-      </c>
-      <c r="C121" t="s">
-        <v>10</v>
+        <v>107</v>
+      </c>
+      <c r="C121" s="2" t="s">
+        <v>6</v>
       </c>
       <c r="D121">
-        <v>-1.998998198445546</v>
+        <v>-0.13718772674175489</v>
       </c>
       <c r="E121">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F121">
-        <v>75</v>
+        <v>66</v>
       </c>
     </row>
     <row r="122" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A122" s="1">
-        <v>24</v>
+        <v>76</v>
       </c>
       <c r="B122" t="s">
-        <v>35</v>
-      </c>
-      <c r="C122" t="s">
-        <v>13</v>
+        <v>83</v>
+      </c>
+      <c r="C122" s="2" t="s">
+        <v>6</v>
       </c>
       <c r="D122">
-        <v>0</v>
+        <v>-0.29438126778694468</v>
       </c>
       <c r="E122">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F122">
-        <v>57</v>
+        <v>67</v>
       </c>
     </row>
     <row r="123" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A123" s="1">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="B123" t="s">
-        <v>47</v>
-      </c>
-      <c r="C123" t="s">
-        <v>10</v>
+        <v>53</v>
+      </c>
+      <c r="C123" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D123">
-        <v>2.6500239639328731</v>
+        <v>-0.34918308632545703</v>
       </c>
       <c r="E123">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F123">
-        <v>97</v>
+        <v>101</v>
       </c>
     </row>
     <row r="124" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A124" s="1">
-        <v>48</v>
+        <v>110</v>
       </c>
       <c r="B124" t="s">
-        <v>59</v>
-      </c>
-      <c r="C124" t="s">
-        <v>10</v>
+        <v>117</v>
+      </c>
+      <c r="C124" s="2" t="s">
+        <v>6</v>
       </c>
       <c r="D124">
-        <v>0</v>
+        <v>-0.44508886589783908</v>
       </c>
       <c r="E124">
         <v>1</v>
       </c>
       <c r="F124">
-        <v>89</v>
+        <v>151</v>
       </c>
     </row>
     <row r="125" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A125" s="1">
-        <v>65</v>
+        <v>28</v>
       </c>
       <c r="B125" t="s">
-        <v>76</v>
-      </c>
-      <c r="C125" t="s">
-        <v>13</v>
+        <v>35</v>
+      </c>
+      <c r="C125" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D125">
-        <v>-0.87105995222732724</v>
+        <v>-0.51980146313749753</v>
       </c>
       <c r="E125">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F125">
-        <v>63</v>
+        <v>75</v>
       </c>
     </row>
     <row r="126" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A126" s="1">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="B126" t="s">
-        <v>103</v>
-      </c>
-      <c r="C126" t="s">
-        <v>13</v>
+        <v>96</v>
+      </c>
+      <c r="C126" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D126">
-        <v>0.83910408072443454</v>
+        <v>-0.61584370402419808</v>
       </c>
       <c r="E126">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F126">
-        <v>93</v>
+        <v>55</v>
       </c>
     </row>
     <row r="127" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A127" s="1">
-        <v>107</v>
+        <v>22</v>
       </c>
       <c r="B127" t="s">
-        <v>118</v>
-      </c>
-      <c r="C127" t="s">
-        <v>13</v>
+        <v>29</v>
+      </c>
+      <c r="C127" s="2" t="s">
+        <v>6</v>
       </c>
       <c r="D127">
-        <v>1.3518348393178721</v>
+        <v>-0.64182248254319685</v>
       </c>
       <c r="E127">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F127">
-        <v>354</v>
+        <v>204</v>
       </c>
     </row>
     <row r="128" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A128" s="1">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B128" t="s">
-        <v>121</v>
-      </c>
-      <c r="C128" t="s">
-        <v>10</v>
+        <v>119</v>
+      </c>
+      <c r="C128" s="2" t="s">
+        <v>6</v>
       </c>
       <c r="D128">
-        <v>-0.44508886589783908</v>
+        <v>-0.66393459056578163</v>
       </c>
       <c r="E128">
-        <v>1</v>
+        <v>7.0000000000000009</v>
       </c>
       <c r="F128">
-        <v>151</v>
+        <v>169</v>
       </c>
     </row>
     <row r="129" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A129" s="1">
-        <v>120</v>
+        <v>65</v>
       </c>
       <c r="B129" t="s">
-        <v>131</v>
-      </c>
-      <c r="C129" t="s">
-        <v>13</v>
+        <v>72</v>
+      </c>
+      <c r="C129" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D129">
-        <v>1.1918215791420561</v>
+        <v>-0.87105995222732724</v>
       </c>
       <c r="E129">
         <v>1</v>
       </c>
       <c r="F129">
-        <v>87</v>
+        <v>63</v>
       </c>
     </row>
     <row r="130" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A130" s="1">
-        <v>8</v>
+        <v>88</v>
       </c>
       <c r="B130" t="s">
-        <v>19</v>
-      </c>
-      <c r="C130" t="s">
-        <v>10</v>
+        <v>95</v>
+      </c>
+      <c r="C130" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="D130">
-        <v>4.6653570953300241</v>
+        <v>-0.87195005133563086</v>
       </c>
       <c r="E130">
-        <v>0.99999999999999989</v>
+        <v>5</v>
       </c>
       <c r="F130">
-        <v>107</v>
+        <v>120</v>
       </c>
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A131" s="1">
-        <v>11</v>
+        <v>68</v>
       </c>
       <c r="B131" t="s">
-        <v>22</v>
-      </c>
-      <c r="C131" t="s">
-        <v>13</v>
+        <v>75</v>
+      </c>
+      <c r="C131" s="2" t="s">
+        <v>6</v>
       </c>
       <c r="D131">
-        <v>0</v>
+        <v>-1.827019897327971</v>
       </c>
       <c r="E131">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F131">
-        <v>93</v>
+        <v>63</v>
       </c>
     </row>
     <row r="132" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A132" s="1">
-        <v>51</v>
+        <v>1</v>
       </c>
       <c r="B132" t="s">
-        <v>62</v>
-      </c>
-      <c r="C132" t="s">
-        <v>10</v>
+        <v>7</v>
+      </c>
+      <c r="C132" s="2" t="s">
+        <v>6</v>
       </c>
       <c r="D132">
-        <v>0</v>
+        <v>-1.998998198445546</v>
       </c>
       <c r="E132">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F132">
-        <v>56</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:F132" xr:uid="{00000000-0001-0000-0100-000000000000}">
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F132">
-      <sortCondition descending="1" ref="E1:E132"/>
+      <sortCondition descending="1" ref="D1:D132"/>
     </sortState>
   </autoFilter>
+  <conditionalFormatting sqref="D1:D1048576">
+    <cfRule type="colorScale" priority="9">
+      <colorScale>
+        <cfvo type="num" val="1"/>
+        <cfvo type="num" val="3"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFE43B34"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C1:C1048576">
+    <cfRule type="endsWith" dxfId="3" priority="3" operator="endsWith" text="Pol I">
+      <formula>RIGHT(C1,LEN("Pol I"))="Pol I"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C2:C132">
+    <cfRule type="endsWith" dxfId="2" priority="2" operator="endsWith" text="Pol II">
+      <formula>RIGHT(C2,LEN("Pol II"))="Pol II"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E2:E132">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF1F8242"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>